<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.003-01 Nina et le gâteau au citron
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.003-01.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.003-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>marché</t>
+          <t>marché, pavés, cagette, citron, gâteau, poire, sac, plateau, miettes, bois</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Au marché, le gâteau au citron n'est plus là. Nina dit qu'elle est déçue. Elle cherche une autre idée. Elle choisit une poire.</t>
+          <t>Un citron échappe aux doigts de maman. Sur le bois, un éclat de cagette luit. Nina veut le gâteau au citron, maintenant. Le plateau est vide. Sourire parti. Trou dans la poitrine. Papa s'accroupit. Nina dit qu'elle est déçue. Merci vécu. Deuxième ruse : poire trop haute, presque prise, autre enfant. Elle refuse de foncer. Elle choisit une poire plus basse. Un éclat de cagette tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les fraises du cageot brillent. Une balance fait ding, tout doux. Le store claque un peu au vent. Ça sent le citron et le pain chaud. Les pavés sont froids sous les chaussures. Un pigeon picore une miette, puis part. Je tiens le sac, Nina. On reste près de moi, d'accord ? D'accord, papa. Tu as vu les citrons jaunes ? Ils sentent fort. Oui. Ils sentent le sucre. En ce moment, Nina veut un gâteau. Un gâteau au citron, tout jaune. Celui-là, papa. On demande, oui. Le plateau est vide. Il reste seulement des miettes. Il n'y en a plus, aujourd'hui. Plus de gâteau... Nina sent ses épaules tomber. Sa gorge se serre un peu. Je suis déçue. Tu es déçue. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Souffle une fois, Nina. Nina souffle une fois. Elle regarde les fruits jaunes. Des pommes. Des citrons. Une poire. Une poire, alors. Une poire. C'est une autre idée. Bravo. Tu as nommé : déçue. Ils achètent une poire juteuse. Nina la tient contre elle. La peau est lisse et froide. Être déçue, ce n'est pas honteux. Une autre idée peut venir. La poire, alors. Oui. La poire. Tu la tiens bien ? Oui. Tout contre moi. Le store claque encore un peu. Les fraises brillent toujours.</t>
+          <t>Un citron échappe aux doigts de maman. Il roule, papa ! Tu le rattrapes, Nina ? Oui, papa. Nina pose le pied devant le fruit jaune. Je l'ai, maman. Il est froid, Nina ? Un peu, maman. Le citron sent fort, près du sac. Ça sent le citron. Tu le sens, toi ? Oui, papa. Maman ouvre une cagette de bois, près des pavés. Elle est en bois. Tu la vois, la cagette ? Oui, maman. Sur le bois, un éclat de cagette luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Le soleil le touche. Nina pose le citron dans la cagette. Il tient. Il est rentré ? Oui, maman. Les pavés du marché sont froids sous les chaussures. Ils sont froids. Tes pieds sont bien, Nina ? Un peu froids. Le sac de papa tape contre sa jambe. Le sac est lourd. Je tiens le sac, Nina. D'accord, maman. Un plateau de gâteaux attend, un peu plus loin. Des gâteaux ! Tu les vois, les jaunes ? Le gâteau au citron. En ce moment, Nina tend les deux mains. Je veux le gâteau, maintenant ! Tout de suite ? Oui, papa. Nina avance trop vite vers le plateau. Ses doigts touchent seulement des miettes. Le plateau est vide, près des citrons. Il n'y en a plus. Le gâteau est parti, Nina ? Oui, maman. Ça sent le citron, même sans gâteau. Le sourire de Nina disparaît. Dans sa poitrine, l'envie du gâteau fait un trou. L'envie et le trou se bousculent sans place. Ses épaules tombent un peu. J'ai mal au ventre. Ta gorge est serrée, Nina ? Un peu, papa. Papa s'accroupit à la même hauteur, sans parler. Tes mains sont chaudes, Nina ? Un peu, maman. Je suis déçue. L'éclat de cagette tremble, puis tient. Nina lève les yeux vers les fruits jaunes. Des citrons. Tu les vois, Nina ? Oui, papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les fraises du cageot brillent. Une balance fait ding, tout doux. Le store claque un peu au vent. Ça sent le citron et le pain chaud. Les pavés sont froids sous les chaussures. Un pigeon picore une miette, puis part. Je tiens le sac, Nina. On reste près de moi, d'accord ? D'accord, papa. Tu as vu les citrons jaunes ? Ils sentent fort. Oui. Ils sentent le sucre. En ce moment, Nina veut un gâteau. Un gâteau au citron, tout jaune. Celui-là, papa. On demande, oui. Le plateau est vide. Il reste seulement des miettes. Il n'y en a plus, aujourd'hui. Plus de gâteau... Nina sent ses épaules tomber. Sa gorge se serre un peu. Je suis déçue. Tu es déçue. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Souffle une fois, Nina. Nina souffle une fois. Elle regarde les fruits jaunes. Des pommes. Des citrons. Une poire. Une poire, alors. Une poire. C'est une autre idée. Bravo. Tu as nommé : déçue. Ils achètent une poire juteuse. Nina la tient contre elle. La peau est lisse et froide. Être déçue, ce n'est pas honteux. Une autre idée peut venir. La poire, alors. Oui. La poire. Tu la tiens bien ? Oui. Tout contre moi. Le store claque encore un peu. Les fraises brillent toujours.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un citron échappe aux doigts de maman. Il roule, papa ! Tu le rattrapes, Nina ? Oui, papa. Nina pose le pied devant le fruit jaune. Je l'ai, maman. Il est froid, Nina ? Un peu, maman. Le citron sent fort, près du sac. Ça sent le citron. Tu le sens, toi ? Oui, papa. Maman ouvre une cagette de bois, près des pavés. Elle est en bois. Tu la vois, la cagette ? Oui, maman. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de cagette&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Le soleil le touche. Nina pose le citron dans la cagette. Il tient. Il est rentré ? Oui, maman. Les pavés du marché sont froids sous les chaussures. Ils sont froids. Tes pieds sont bien, Nina ? Un peu froids. Le sac de papa tape contre sa jambe. Le sac est lourd. Je tiens le sac, Nina. D'accord, maman. Un plateau de gâteaux attend, un peu plus loin. Des gâteaux ! Tu les vois, les jaunes ? Le gâteau au citron. En ce moment, Nina tend les deux mains. Je veux le gâteau, maintenant ! Tout de suite ? Oui, papa. Nina avance trop vite vers le plateau. Ses doigts touchent seulement des miettes. Le plateau est vide, près des citrons. Il n'y en a plus. Le gâteau est parti, Nina ? Oui, maman. Ça sent le citron, même sans gâteau. Le sourire de Nina disparaît. Dans sa poitrine, l'envie du gâteau fait un trou. L'envie et le trou se bousculent sans place. Ses épaules tombent un peu. J'ai mal au ventre. Ta gorge est serrée, Nina ? Un peu, papa. Papa s'accroupit à la même hauteur, sans parler. Tes mains sont chaudes, Nina ? Un peu, maman. Je suis déçue. L'éclat de cagette tremble, puis tient. Nina lève les yeux vers les fruits jaunes. Des citrons. Tu les vois, Nina ? Oui, papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sami marche au marché, la main dans la main de papa. Il sent l'odeur du citron. Il veut un gâteau au citron. Le marchand secoue la tête. Il dit : il n'y en a plus aujourd'hui. Sami sent ses épaules tomber. Sa gorge se serre un peu. Sami dit : je suis &lt;emphasis&gt;déçu&lt;/emphasis&gt;. Papa s'accroupit. Papa dit : un souhait peut attendre. On peut chercher une autre idée. Sami souffle une fois. Il regarde les fruits jaunes. Il dit : une poire, alors. Papa sourit. Ils achètent une poire juteuse. Sami la tient contre lui. Être déçu, ce n'est pas honteux. Une autre idée peut venir. [pause]</t>
+          <t>Un citron échappe aux doigts de maman. Il roule, papa ! Tu le rattrapes, Nina ? Oui, papa. Nina pose le pied devant le fruit jaune. Je l'ai, maman. Il est froid, Nina ? Un peu, maman. Le citron sent fort, près du sac. Ça sent le citron. Tu le sens, toi ? Oui, papa. Maman ouvre une cagette de bois, près des pavés. Elle est en bois. Tu la vois, la cagette ? Oui, maman. Sur le bois, un &lt;emphasis&gt;éclat de cagette&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Le soleil le touche. Nina pose le citron dans la cagette. Il tient. Il est rentré ? Oui, maman. Les pavés du marché sont froids sous les chaussures. Ils sont froids. Tes pieds sont bien, Nina ? Un peu froids. Le sac de papa tape contre sa jambe. Le sac est lourd. Je tiens le sac, Nina. D'accord, maman. Un plateau de gâteaux attend, un peu plus loin. Des gâteaux ! Tu les vois, les jaunes ? Le gâteau au citron. En ce moment, Nina tend les deux mains. Je veux le gâteau, maintenant ! Tout de suite ? Oui, papa. Nina avance trop vite vers le plateau. Ses doigts touchent seulement des miettes. Le plateau est vide, près des citrons. Il n'y en a plus. Le gâteau est parti, Nina ? Oui, maman. Ça sent le citron, même sans gâteau. Le sourire de Nina disparaît. Dans sa poitrine, l'envie du gâteau fait un trou. L'envie et le trou se bousculent sans place. Ses épaules tombent un peu. J'ai mal au ventre. Ta gorge est serrée, Nina ? Un peu, papa. Papa s'accroupit à la même hauteur, sans parler. Tes mains sont chaudes, Nina ? Un peu, maman. Je suis déçue. L'éclat de cagette tremble, puis tient. Nina lève les yeux vers les fruits jaunes. Des citrons. Tu les vois, Nina ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>éclat de cagette</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,53 +1321,82 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis déception; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_gateau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les fraises du cageot brillent.
-narrateur|Une balance fait ding, tout doux.
-narrateur|Le store claque un peu au vent.
-narrateur|Ça sent le citron et le pain chaud.
-narrateur|Les pavés sont froids sous les chaussures.
-narrateur|Un pigeon picore une miette, puis part.
+          <t>narrateur|Un citron échappe aux doigts de maman.
+enfant-f|Il roule, papa !
+papa|Tu le rattrapes, Nina ?
+enfant-f|Oui, papa.
+narrateur|Nina pose le pied devant le fruit jaune.
+enfant-f|Je l'ai, maman.
+maman|Il est froid, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Le citron sent fort, près du sac.
+enfant-f|Ça sent le citron.
+papa|Tu le sens, toi ?
+enfant-f|Oui, papa.
+narrateur|Maman ouvre une cagette de bois, près des pavés.
+enfant-f|Elle est en bois.
+maman|Tu la vois, la cagette ?
+enfant-f|Oui, maman.
+narrateur|Sur le bois, un éclat de cagette luit.
+enfant-f|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+papa|Le soleil le touche.
+narrateur|Nina pose le citron dans la cagette.
+enfant-f|Il tient.
+maman|Il est rentré ?
+enfant-f|Oui, maman.
+narrateur|Les pavés du marché sont froids sous les chaussures.
+enfant-f|Ils sont froids.
+papa|Tes pieds sont bien, Nina ?
+enfant-f|Un peu froids.
+narrateur|Le sac de papa tape contre sa jambe.
+enfant-f|Le sac est lourd.
 maman|Je tiens le sac, Nina.
-papa|On reste près de moi, d'accord ?
-enfant-f|D'accord, papa.
-maman|Tu as vu les citrons jaunes ?
-enfant-f|Ils sentent fort.
-papa|Oui. Ils sentent le sucre.
-narrateur|En ce moment, Nina veut un gâteau.
-narrateur|Un gâteau au citron, tout jaune.
-enfant-f|Celui-là, papa.
-papa|On demande, oui.
-narrateur|Le plateau est vide.
-narrateur|Il reste seulement des miettes.
-narrateur|Il n'y en a plus, aujourd'hui.
-enfant-f|Plus de gâteau...
-narrateur|Nina sent ses épaules tomber.
-narrateur|Sa gorge se serre un peu.
+enfant-f|D'accord, maman.
+narrateur|Un plateau de gâteaux attend, un peu plus loin.
+enfant-f|Des gâteaux !
+papa|Tu les vois, les jaunes ?
+enfant-f|Le gâteau au citron.
+narrateur|En ce moment, Nina tend les deux mains.
+enfant-f|Je veux le gâteau, maintenant !
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|Nina avance trop vite vers le plateau.
+narrateur|Ses doigts touchent seulement des miettes.
+narrateur|Le plateau est vide, près des citrons.
+enfant-f|Il n'y en a plus.
+maman|Le gâteau est parti, Nina ?
+enfant-f|Oui, maman.
+narrateur|Ça sent le citron, même sans gâteau.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie du gâteau fait un trou.
+narrateur|L'envie et le trou se bousculent sans place.
+narrateur|Ses épaules tombent un peu.
+enfant-f|J'ai mal au ventre.
+papa|Ta gorge est serrée, Nina ?
+enfant-f|Un peu, papa.
+narrateur|Papa s'accroupit à la même hauteur, sans parler.
+maman|Tes mains sont chaudes, Nina ?
+enfant-f|Un peu, maman.
 enfant-f|Je suis déçue.
-papa|Tu es déçue. Ce n'est pas honteux.
-papa|Un souhait peut attendre.
-papa|On peut chercher une autre idée.
-maman|Souffle une fois, Nina.
-narrateur|Nina souffle une fois.
-narrateur|Elle regarde les fruits jaunes.
-narrateur|Des pommes. Des citrons. Une poire.
-enfant-f|Une poire, alors.
-papa|Une poire. C'est une autre idée.
-maman|Bravo. Tu as nommé : déçue.
-narrateur|Ils achètent une poire juteuse.
-narrateur|Nina la tient contre elle.
-narrateur|La peau est lisse et froide.
-papa|Être déçue, ce n'est pas honteux.
-papa|Une autre idée peut venir.
-enfant-f|La poire, alors.
-maman|Oui. La poire.
-papa|Tu la tiens bien ?
-enfant-f|Oui. Tout contre moi.
-narrateur|Le store claque encore un peu.
-narrateur|Les fraises brillent toujours.</t>
+narrateur|L'éclat de cagette tremble, puis tient.
+narrateur|Nina lève les yeux vers les fruits jaunes.
+enfant-f|Des citrons.
+papa|Tu les vois, Nina ?
+enfant-f|Oui, papa.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>marché,citron</t>
         </is>
       </c>
     </row>
@@ -1399,12 +1428,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le gâteau n'est plus là. Que dit Nina ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le gâteau n'est plus là. Que dit &lt;emphasis level="moderate"&gt;Nina&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le gâteau n'est plus là. Que dit Sami ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le gâteau n'est plus là. Que dit &lt;emphasis&gt;Nina&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1429,7 +1458,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Sami cherche une autre idée. Que dit-il d'abord ?</t>
+          <t>Nina cherche une autre idée. Que dit-elle d'abord ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1467,7 +1496,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1478,7 +1507,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1493,34 +1522,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Nina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1535,22 +1568,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_gateau_n_est_plus_la_que_dit_nina; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Le gâteau n'est plus là. Que dit Nina ?</t>
+          <t>narrateur|Le gâteau n'est plus là.
+narrateur|Que dit Nina ?</t>
         </is>
       </c>
     </row>
@@ -1577,17 +1611,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina tient encore la poire. Je suis déçue. Oui. Et une autre idée est arrivée. Le souhait peut attendre. Bravo. Tu as dit ce que tu sentais. Tu as choisi la poire ? Oui. La poire. Papa range le sac. Ça sent encore le citron.</t>
+          <t>Nina reste près de la cagette, un moment. Le gâteau, maintenant. Les mots se bousculent dans sa bouche. Je le prends. Nina avance les mains, trop vite. Puis elle s'arrête. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les fruits, un instant. Elle écoute le marché, près des pavés. Tu restes un peu, Nina ? Oui, papa. Merci, Nina. Papa reste à la même hauteur. Le citron est froid, sous les doigts. Il est lisse. La poitrine de Nina ralentit un peu. Les épaules se relèvent un peu. Une poire, alors. Tu la vois, la poire ? Oui, maman. Elle est jaune, Nina ? Un peu verte. Nina tend le doigt vers une poire. Celle-là. Tes joues sont chaudes, Nina ? Un peu, maman. Le ventre de Nina se desserre. On s'approche sans se presser ? Oui. Ils se lèvent, sans se bousculer. La poire, papa. On y va, sans se presser.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina tient encore la poire. Je suis déçue. Oui. Et une autre idée est arrivée. Le souhait peut attendre. Bravo. Tu as dit ce que tu sentais. Tu as choisi la poire ? Oui. La poire. Papa range le sac. Ça sent encore le citron.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina reste près de la cagette, un moment. Le gâteau, maintenant. Les mots se bousculent dans sa bouche. Je le prends. Nina avance les mains, trop vite. Puis elle s'arrête. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les fruits, un instant. Elle écoute le marché, près des pavés. Tu restes un peu, Nina ? Oui, papa. Merci, Nina. Papa reste à la même hauteur. Le citron est froid, sous les doigts. Il est lisse. La poitrine de Nina ralentit un peu. Les épaules se relèvent un peu. Une &lt;emphasis level="moderate"&gt;poire&lt;/emphasis&gt;, alors. Tu la vois, la poire ? Oui, maman. Elle est jaune, Nina ? Un peu verte. Nina tend le doigt vers une poire. Celle-là. Tes joues sont chaudes, Nina ? Un peu, maman. Le ventre de Nina se desserre. On s'approche sans se presser ? Oui. Ils se lèvent, sans se bousculer. La poire, papa. On y va, sans se presser.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sami a nommé : &lt;emphasis&gt;déçu&lt;/emphasis&gt;. Le souhait peut attendre. Une autre idée est arrivée. [pause]</t>
+          <t>Nina reste près de la cagette, un moment. Le gâteau, maintenant. Les mots se bousculent dans sa bouche. Je le prends. Nina avance les mains, trop vite. Puis elle s'arrête. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les fruits, un instant. Elle écoute le marché, près des pavés. Tu restes un peu, Nina ? Oui, papa. Merci, Nina. Papa reste à la même hauteur. Le citron est froid, sous les doigts. Il est lisse. La poitrine de Nina ralentit un peu. Les épaules se relèvent un peu. Une &lt;emphasis&gt;poire&lt;/emphasis&gt;, alors. Tu la vois, la poire ? Oui, maman. Elle est jaune, Nina ? Un peu verte. Nina tend le doigt vers une poire. Celle-là. Tes joues sont chaudes, Nina ? Un peu, maman. Le ventre de Nina se desserre. On s'approche sans se presser ? Oui. Ils se lèvent, sans se bousculer. La poire, papa. On y va, sans se presser. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1634,7 +1668,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1642,10 +1676,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1668,30 +1702,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>poire</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1700,10 +1734,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1716,20 +1750,50 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis soulagement; intensite=2; destinataire=enfant; sous_texte=elle_dit_une_poire_sans_slogan; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina tient encore la poire.
-enfant-f|Je suis déçue.
-papa|Oui. Et une autre idée est arrivée.
-maman|Le souhait peut attendre.
-papa|Bravo. Tu as dit ce que tu sentais.
-papa|Tu as choisi la poire ?
-enfant-f|Oui. La poire.
-narrateur|Papa range le sac.
-narrateur|Ça sent encore le citron.</t>
+          <t>narrateur|Nina reste près de la cagette, un moment.
+enfant-f|Le gâteau, maintenant.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Je le prends.
+narrateur|Nina avance les mains, trop vite.
+narrateur|Puis elle s'arrête.
+narrateur|Nina refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe les fruits, un instant.
+narrateur|Elle écoute le marché, près des pavés.
+papa|Tu restes un peu, Nina ?
+enfant-f|Oui, papa.
+papa|Merci, Nina.
+narrateur|Papa reste à la même hauteur.
+maman|Le citron est froid, sous les doigts.
+enfant-f|Il est lisse.
+narrateur|La poitrine de Nina ralentit un peu.
+narrateur|Les épaules se relèvent un peu.
+enfant-f|Une poire, alors.
+maman|Tu la vois, la poire ?
+enfant-f|Oui, maman.
+papa|Elle est jaune, Nina ?
+enfant-f|Un peu verte.
+narrateur|Nina tend le doigt vers une poire.
+enfant-f|Celle-là.
+maman|Tes joues sont chaudes, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Nina se desserre.
+papa|On s'approche sans se presser ?
+enfant-f|Oui.
+narrateur|Ils se lèvent, sans se bousculer.
+enfant-f|La poire, papa.
+papa|On y va, sans se presser.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>marché</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nina croque la poire. Le jus est sucré sur ses lèvres. Elle est juteuse ? Oui. Sucrée. On rentre quand tu es prête ? Encore un bout. On reste. Tu as trouvé une autre idée. Je suis moins déçue. La poire est là. Papa range le sac. Ils rentrent à la maison.</t>
+          <t>Nina lève la main vers la poire. Je la prends ! Un enfant plus grand tend la main vers la poire. La poire bascule au bord, trop haute. Elle part ! La poire est presque prise, au-dessus des doigts. Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la poire, un instant. Elle écoute le marché, près de la cagette. Sur le bois, un éclat de cagette luit. Là, sur le bois. Tu vois le point, Nina ? Oui, papa. L'enfant plus grand prend la poire trop haute. Pas celle-là. Tu en vois une autre, Nina ? Plus bas. Une poire plus basse attend à hauteur de main. Celle-là, maman. Tu la prends, Nina ? Oui, papa. Nina détache la poire plus basse, sans se presser. La peau est lisse et froide. Elle est lourde. Elle tient dans ta main ? Oui, maman. Nina la serre contre elle. Ma poire. Elle a une petite trace, Nina. Elle a failli partir. La poire sent le sucre, un peu. Et le citron, autour. On reste près de la cagette ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nina croque la poire. Le jus est sucré sur ses lèvres. Elle est juteuse ? Oui. Sucrée. On rentre quand tu es prête ? Encore un bout. On reste. Tu as trouvé une autre idée. Je suis moins déçue. La poire est là. Papa range le sac. Ils rentrent à la maison.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina lève la main vers la poire. Je la prends ! Un enfant plus grand tend la main vers la poire. La poire bascule au bord, trop haute. Elle part ! La poire est presque prise, au-dessus des doigts. Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la poire, un instant. Elle écoute le marché, près de la cagette. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de cagette&lt;/emphasis&gt; luit. Là, sur le bois. Tu vois le point, Nina ? Oui, papa. L'enfant plus grand prend la poire trop haute. Pas celle-là. Tu en vois une autre, Nina ? Plus bas. Une poire plus basse attend à hauteur de main. Celle-là, maman. Tu la prends, Nina ? Oui, papa. Nina détache la poire plus basse, sans se presser. La peau est lisse et froide. Elle est lourde. Elle tient dans ta main ? Oui, maman. Nina la serre contre elle. Ma poire. Elle a une petite trace, Nina. Elle a failli partir. La poire sent le sucre, un peu. Et le citron, autour. On reste près de la cagette ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sami croque la poire. Papa range le sac. Ils rentrent à la maison. [pause]</t>
+          <t>Nina lève la main vers la poire. Je la prends ! Un enfant plus grand tend la main vers la poire. La poire bascule au bord, trop haute. Elle part ! La poire est presque prise, au-dessus des doigts. Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la poire, un instant. Elle écoute le marché, près de la cagette. Sur le bois, un &lt;emphasis&gt;éclat de cagette&lt;/emphasis&gt; luit. Là, sur le bois. Tu vois le point, Nina ? Oui, papa. L'enfant plus grand prend la poire trop haute. Pas celle-là. Tu en vois une autre, Nina ? Plus bas. Une poire plus basse attend à hauteur de main. Celle-là, maman. Tu la prends, Nina ? Oui, papa. Nina détache la poire plus basse, sans se presser. La peau est lisse et froide. Elle est lourde. Elle tient dans ta main ? Oui, maman. Nina la serre contre elle. Ma poire. Elle a une petite trace, Nina. Elle a failli partir. La poire sent le sucre, un peu. Et le citron, autour. On reste près de la cagette ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1813,7 +1877,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1821,10 +1885,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1845,28 +1909,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cagette</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1875,10 +1943,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1889,20 +1957,56 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=poire_presque_prise_trop_haute_autre_enfant; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nina croque la poire.
-narrateur|Le jus est sucré sur ses lèvres.
-maman|Elle est juteuse ?
-enfant-f|Oui. Sucrée.
-maman|On rentre quand tu es prête ?
-enfant-f|Encore un bout.
-papa|On reste. Tu as trouvé une autre idée.
-enfant-f|Je suis moins déçue.
-maman|La poire est là.
-narrateur|Papa range le sac.
-narrateur|Ils rentrent à la maison.</t>
+          <t>narrateur|Nina lève la main vers la poire.
+enfant-f|Je la prends !
+narrateur|Un enfant plus grand tend la main vers la poire.
+narrateur|La poire bascule au bord, trop haute.
+enfant-f|Elle part !
+narrateur|La poire est presque prise, au-dessus des doigts.
+narrateur|Nina avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe la poire, un instant.
+narrateur|Elle écoute le marché, près de la cagette.
+narrateur|Sur le bois, un éclat de cagette luit.
+enfant-f|Là, sur le bois.
+papa|Tu vois le point, Nina ?
+enfant-f|Oui, papa.
+narrateur|L'enfant plus grand prend la poire trop haute.
+enfant-f|Pas celle-là.
+maman|Tu en vois une autre, Nina ?
+enfant-f|Plus bas.
+narrateur|Une poire plus basse attend à hauteur de main.
+enfant-f|Celle-là, maman.
+papa|Tu la prends, Nina ?
+enfant-f|Oui, papa.
+narrateur|Nina détache la poire plus basse, sans se presser.
+narrateur|La peau est lisse et froide.
+enfant-f|Elle est lourde.
+maman|Elle tient dans ta main ?
+enfant-f|Oui, maman.
+narrateur|Nina la serre contre elle.
+enfant-f|Ma poire.
+papa|Elle a une petite trace, Nina.
+enfant-f|Elle a failli partir.
+narrateur|La poire sent le sucre, un peu.
+enfant-f|Et le citron, autour.
+papa|On reste près de la cagette ?
+enfant-f|Oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>marché,poire</t>
         </is>
       </c>
     </row>
@@ -1929,17 +2033,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Un souhait peut attendre. Bravo, Nina.</t>
+          <t>Ils restent près de la cagette. Maman essuie un peu de jus sur le bois. La poire a une trace, papa. Tu l'as vue, toi ? Oui, près du bord. On est bien, ici. Nina tapote le bois de la cagette. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La poire est restée, Nina. Oui, avec nous. Ça sent le citron, un peu tiède. Et le bois, maman. Oui, dans l'air. Le marché sent le sucre, Nina ? Oui, papa. La poire reste contre le sac. Un éclat de cagette tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Un souhait peut attendre. Bravo, Nina.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la cagette. Maman essuie un peu de jus sur le bois. La poire a une trace, papa. Tu l'as vue, toi ? Oui, près du bord. On est bien, ici. Nina tapote le bois de la cagette. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La poire est restée, Nina. Oui, avec nous. Ça sent le citron, un peu tiède. Et le bois, maman. Oui, dans l'air. Le marché sent le sucre, Nina ? Oui, papa. La poire reste contre le sac. Un &lt;emphasis level="moderate"&gt;éclat de cagette&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la cagette. Maman essuie un peu de jus sur le bois. La poire a une trace, papa. Tu l'as vue, toi ? Oui, près du bord. On est bien, ici. Nina tapote le bois de la cagette. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La poire est restée, Nina. Oui, avec nous. Ça sent le citron, un peu tiède. Et le bois, maman. Oui, dans l'air. Le marché sent le sucre, Nina ? Oui, papa. La poire reste contre le sac. Un &lt;emphasis&gt;éclat de cagette&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1986,7 +2090,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -1994,10 +2098,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2006,12 +2110,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2020,17 +2124,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cagette</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2039,11 +2147,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2052,27 +2160,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_soulagement; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit : je suis déçue.
-enfant-f|J'ai trouvé une autre idée.
-papa|Un souhait peut attendre.
-maman|Bravo, Nina.</t>
+          <t>narrateur|Ils restent près de la cagette.
+narrateur|Maman essuie un peu de jus sur le bois.
+enfant-f|La poire a une trace, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, près du bord.
+maman|On est bien, ici.
+narrateur|Nina tapote le bois de la cagette.
+enfant-f|Il a une trace de jus.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|La poire est restée, Nina.
+enfant-f|Oui, avec nous.
+narrateur|Ça sent le citron, un peu tiède.
+enfant-f|Et le bois, maman.
+maman|Oui, dans l'air.
+papa|Le marché sent le sucre, Nina ?
+enfant-f|Oui, papa.
+narrateur|La poire reste contre le sac.
+narrateur|Un éclat de cagette tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2143,6 +2270,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>